<commit_message>
Added interpretation of first two Graphs
</commit_message>
<xml_diff>
--- a/WebsiteVorschau/Visulisation/Testdaten.xlsx
+++ b/WebsiteVorschau/Visulisation/Testdaten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fhooe-my.sharepoint.com/personal/s2310307083_fhooe_at/Documents/Hagenberg/Bachelorarbeit2025-26/WebsiteVorschau/Visulisation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="8_{D010FF73-5F9C-4556-962E-81E5C6D0207B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5215489A-6C1A-4537-AA4E-D6ED0FCB8645}"/>
+  <xr:revisionPtr revIDLastSave="299" documentId="8_{D010FF73-5F9C-4556-962E-81E5C6D0207B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF2DD25-BA2C-4696-9192-B94F3FEBA049}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{587AFEF8-2E2A-4687-9884-DC36B90FBF70}"/>
+    <workbookView xWindow="28680" yWindow="-6720" windowWidth="29040" windowHeight="15720" xr2:uid="{587AFEF8-2E2A-4687-9884-DC36B90FBF70}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1783,15 +1783,15 @@
         <v>4703</v>
       </c>
       <c r="AD12">
-        <f t="shared" ref="AD12:AD13" si="0">AVERAGE(E12:AC12)</f>
+        <f>AVERAGE(E12:AC12)</f>
         <v>4658.5200000000004</v>
       </c>
       <c r="AE12">
-        <f t="shared" ref="AE12:AE13" si="1">MEDIAN(E12:AC12)</f>
+        <f t="shared" ref="AE12:AE13" si="0">MEDIAN(E12:AC12)</f>
         <v>4650</v>
       </c>
       <c r="AF12" s="5">
-        <f t="shared" ref="AF12" si="2">_xlfn.STDEV.S(E12:AC12)</f>
+        <f t="shared" ref="AF12" si="1">_xlfn.STDEV.S(E12:AC12)</f>
         <v>45.398347987564492</v>
       </c>
     </row>
@@ -1884,11 +1884,11 @@
         <v>4764</v>
       </c>
       <c r="AD13">
+        <f t="shared" ref="AD12:AD13" si="2">AVERAGE(E13:AC13)</f>
+        <v>4768.6400000000003</v>
+      </c>
+      <c r="AE13">
         <f t="shared" si="0"/>
-        <v>4768.6400000000003</v>
-      </c>
-      <c r="AE13">
-        <f t="shared" si="1"/>
         <v>4764</v>
       </c>
       <c r="AF13" s="5">

</xml_diff>

<commit_message>
Finish Chapter tests no corr
</commit_message>
<xml_diff>
--- a/WebsiteVorschau/Visulisation/Testdaten.xlsx
+++ b/WebsiteVorschau/Visulisation/Testdaten.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="299" documentId="8_{D010FF73-5F9C-4556-962E-81E5C6D0207B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF2DD25-BA2C-4696-9192-B94F3FEBA049}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-6720" windowWidth="29040" windowHeight="15720" xr2:uid="{587AFEF8-2E2A-4687-9884-DC36B90FBF70}"/>
+    <workbookView xWindow="38280" yWindow="3615" windowWidth="29040" windowHeight="15720" xr2:uid="{587AFEF8-2E2A-4687-9884-DC36B90FBF70}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1884,7 +1884,7 @@
         <v>4764</v>
       </c>
       <c r="AD13">
-        <f t="shared" ref="AD12:AD13" si="2">AVERAGE(E13:AC13)</f>
+        <f t="shared" ref="AD13" si="2">AVERAGE(E13:AC13)</f>
         <v>4768.6400000000003</v>
       </c>
       <c r="AE13">

</xml_diff>